<commit_message>
Update API test cases and Postman collection
</commit_message>
<xml_diff>
--- a/api测试用例.xlsx
+++ b/api测试用例.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\22405\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\测试项目\restful-booker-api-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -131,7 +131,7 @@
     <t>接口应按照需求/接口规范对 totalprice 的数据类型进行校验，并返回符合规范的处理结果。</t>
   </si>
   <si>
-    <t>POST 返回 200 OK，响应中的 totalprice 为 null；使用 GET /booking/{bookingid} 查询后，totalprice 仍为 null。</t>
+    <t>POST 返回 200 OK，响应中的 totalprice 为 null。</t>
   </si>
   <si>
     <t>待确认</t>
@@ -425,7 +425,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -441,12 +441,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -858,7 +852,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
@@ -882,16 +876,16 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="13">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="13">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14">
@@ -900,89 +894,89 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="15">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1004,9 +998,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1016,17 +1007,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1426,324 +1411,324 @@
       <c r="J2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" ht="86.4" spans="1:11">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" ht="158.4" spans="1:11">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="K4" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" ht="28.8" spans="1:11">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="11"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="9"/>
     </row>
     <row r="6" ht="28.8" spans="1:11">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="11"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="9"/>
     </row>
     <row r="7" ht="28.8" spans="1:11">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="11"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="8" ht="28.8" spans="1:11">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="11"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="9"/>
     </row>
     <row r="9" ht="28.8" spans="1:11">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="11"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="9"/>
     </row>
     <row r="10" ht="28.8" spans="1:11">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="11"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="9"/>
     </row>
     <row r="11" ht="28.8" spans="1:11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="11"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="9"/>
     </row>
     <row r="12" ht="28.8" spans="1:11">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="11"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="9"/>
     </row>
     <row r="13" ht="28.8" spans="1:11">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="11"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="9"/>
     </row>
     <row r="14" ht="28.8" spans="1:11">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="11"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="9"/>
     </row>
     <row r="15" ht="28.8" spans="1:11">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="11"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="9"/>
     </row>
     <row r="16" ht="28.8" spans="1:11">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="11"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="9"/>
     </row>
     <row r="17" ht="28.8" spans="1:11">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="11"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="9"/>
     </row>
     <row r="18" ht="28.8" spans="1:11">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="11"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="9"/>
     </row>
     <row r="19" ht="28.8" spans="1:11">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="9"/>
     </row>
     <row r="20" ht="28.8" spans="1:11">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="9"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add complete API test cases
</commit_message>
<xml_diff>
--- a/api测试用例.xlsx
+++ b/api测试用例.xlsx
@@ -5,15 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\测试项目\restful-booker-api-testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\22405\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21408" windowHeight="9744"/>
+    <workbookView windowWidth="18600" windowHeight="9744"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="API测试用例" sheetId="1" r:id="rId1"/>
+    <sheet name="执行说明" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">API测试用例!$A$1:$K$35</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -32,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="247">
   <si>
     <t>用例编号</t>
   </si>
@@ -100,128 +104,748 @@
     <t>Pass / Fail</t>
   </si>
   <si>
+    <t>API-HEALTH-001</t>
+  </si>
+  <si>
+    <t>检查服务是否正常运行</t>
+  </si>
+  <si>
+    <t>服务健康检查</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>GET /ping</t>
+  </si>
+  <si>
+    <t>Restful Booker 服务可访问</t>
+  </si>
+  <si>
+    <t>1. 发送 GET /ping 请求
+2. 查看 HTTP 状态码和响应内容</t>
+  </si>
+  <si>
+    <t>无</t>
+  </si>
+  <si>
+    <t>服务正常时返回成功状态（通常为 201 Created）；无业务数据返回要求。</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>API-GET-001</t>
+  </si>
+  <si>
+    <t>查询全部 Booking ID</t>
+  </si>
+  <si>
+    <t>Booking查询</t>
+  </si>
+  <si>
+    <t>GET /booking</t>
+  </si>
+  <si>
+    <t>服务可访问</t>
+  </si>
+  <si>
+    <t>1. 发送 GET /booking 请求
+2. 查看状态码及响应 JSON
+3. 检查返回结构</t>
+  </si>
+  <si>
+    <t>返回成功状态；响应为 Booking ID 列表，每项包含 bookingid。若环境数据变化，列表数量不固定。</t>
+  </si>
+  <si>
+    <t>API-GET-002</t>
+  </si>
+  <si>
+    <t>按有效 ID 查询 Booking</t>
+  </si>
+  <si>
+    <t>GET /booking/{id}</t>
+  </si>
+  <si>
+    <t>存在有效 bookingid；可先创建数据</t>
+  </si>
+  <si>
+    <t>1. 创建一条 Booking 或选取已存在 ID
+2. 发送 GET /booking/{id}
+3. 对比响应字段与创建数据</t>
+  </si>
+  <si>
+    <t>有效 bookingid，例如创建接口返回的 bookingid</t>
+  </si>
+  <si>
+    <t>返回 200 OK；响应包含 firstname、lastname、totalprice、depositpaid、bookingdates 等字段，数据与该记录一致。</t>
+  </si>
+  <si>
+    <t>API-GET-003</t>
+  </si>
+  <si>
+    <t>查询不存在的 Booking ID</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>1. 发送 GET /booking/99999999
+2. 查看状态码及响应体</t>
+  </si>
+  <si>
+    <t>不存在的正整数 ID：99999999</t>
+  </si>
+  <si>
+    <t>返回 404 Not Found；不应返回其他 Booking 的数据。</t>
+  </si>
+  <si>
+    <t>API-GET-004</t>
+  </si>
+  <si>
+    <t>查询 ID 为非数字的 Booking</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>1. 发送 GET /booking/abc
+2. 查看状态码及响应体</t>
+  </si>
+  <si>
+    <t>id=abc</t>
+  </si>
+  <si>
+    <t>请求应被拒绝或返回未找到响应；不得返回无关记录，结果应符合接口实际规范。</t>
+  </si>
+  <si>
+    <t>API-GET-005</t>
+  </si>
+  <si>
+    <t>按姓名过滤 Booking</t>
+  </si>
+  <si>
+    <t>GET /booking?firstname=Tom&amp;lastname=Smith</t>
+  </si>
+  <si>
+    <t>存在符合筛选条件的数据</t>
+  </si>
+  <si>
+    <t>1. 发送带 firstname、lastname 查询参数的 GET 请求
+2. 检查返回 ID 列表
+3. 对列表中的 ID 逐条查询并核对姓名</t>
+  </si>
+  <si>
+    <t>firstname=Tom；lastname=Smith</t>
+  </si>
+  <si>
+    <t>返回符合筛选条件的 Booking ID 列表；结果中的记录应匹配指定姓名。若没有匹配数据，允许返回空列表。</t>
+  </si>
+  <si>
+    <t>API-GET-006</t>
+  </si>
+  <si>
+    <t>按入住日期过滤 Booking</t>
+  </si>
+  <si>
+    <t>GET /booking?checkin=2026-10-02&amp;checkout=2026-10-05</t>
+  </si>
+  <si>
+    <t>服务可访问；筛选日期有效</t>
+  </si>
+  <si>
+    <t>1. 发送带 checkin、checkout 参数的 GET 请求
+2. 检查响应状态和结果
+3. 对返回 ID 核对日期范围</t>
+  </si>
+  <si>
+    <t>checkin=2026-10-02；checkout=2026-10-05</t>
+  </si>
+  <si>
+    <t>返回符合日期筛选条件的 Booking ID 列表；无匹配数据时可返回空列表。</t>
+  </si>
+  <si>
+    <t>API-GET-007</t>
+  </si>
+  <si>
+    <t>查询时传入不存在的姓名</t>
+  </si>
+  <si>
+    <t>GET /booking?firstname=NoSuchName987</t>
+  </si>
+  <si>
+    <t>1. 发送带不存在姓名的查询请求
+2. 检查返回结果</t>
+  </si>
+  <si>
+    <t>firstname=NoSuchName987</t>
+  </si>
+  <si>
+    <t>返回成功状态及空 ID 列表，不应返回不匹配的数据。</t>
+  </si>
+  <si>
     <t>API-POST-001</t>
   </si>
   <si>
-    <t>创建Booking时，totalprice传入字符串类型</t>
+    <t>创建 Booking 时提交完整合法数据</t>
   </si>
   <si>
     <t>Booking创建</t>
   </si>
   <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>post</t>
-  </si>
-  <si>
-    <t>打开测试软件</t>
-  </si>
-  <si>
-    <t>1. 发送 POST /booking 请求
-2. 在请求 Body 中将 totalprice 设置为 "abc"
-3. 点击 Send 发送请求
-4. 查看接口返回结果
-5. 使用 GET /booking/{bookingid} 查询创建的数据</t>
-  </si>
-  <si>
-    <t>"totalprice": "abc"</t>
-  </si>
-  <si>
-    <t>接口应按照需求/接口规范对 totalprice 的数据类型进行校验，并返回符合规范的处理结果。</t>
-  </si>
-  <si>
-    <t>POST 返回 200 OK，响应中的 totalprice 为 null。</t>
-  </si>
-  <si>
-    <t>待确认</t>
+    <t>POST /booking</t>
+  </si>
+  <si>
+    <t>服务可访问；请求头 Content-Type 为 application/json</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 查看状态码和响应体
+3. 获取 bookingid
+4. 使用 GET /booking/{id} 查询并核对字段</t>
+  </si>
+  <si>
+    <t>{"firstname":"Tom","lastname":"Smith","totalprice":100,"depositpaid":true,"bookingdates":{"checkin":"2026-10-02","checkout":"2026-10-05"},"additionalneeds":"Breakfast"}</t>
+  </si>
+  <si>
+    <t>返回创建成功状态（通常为 200 OK）并返回 bookingid；查询新记录时各字段与提交值一致。</t>
   </si>
   <si>
     <t>API-POST-002</t>
   </si>
   <si>
-    <t>创建 Booking 时，POST 请求能够正确创建数据</t>
-  </si>
-  <si>
-    <t>p0</t>
-  </si>
-  <si>
-    <t>1. 发送 POST /booking 请求
-2. 在 Body 中填写完整且合法的 Booking 数据
-3. 点击 Send 发送请求
-4. 查看接口响应
-5. 根据返回的 bookingid 使用 GET /booking/{bookingid} 查询数据
-6. 对比创建时提交的数据与查询返回的数据</t>
-  </si>
-  <si>
-    <t>{
-  "firstname": "Tom",
-  "lastname": "Smith",
-  "totalprice": 100,
-  "depositpaid": true,
-  "bookingdates": {
-    "checkin": "2026-10-02",
-    "checkout": "2026-10-05"
-  },
-  "additionalneeds": "Breakfast"
-}</t>
-  </si>
-  <si>
-    <t>接口返回 200 OK，并返回有效的 bookingid；使用 GET 查询该 bookingid 时，能够正确返回刚才提交的 Booking 数据，数据内容与提交的数据一致。</t>
-  </si>
-  <si>
-    <t>POST 返回 200 OK，并返回 bookingid；使用 GET 查询后，Booking 数据与提交的数据一致。</t>
-  </si>
-  <si>
-    <t>Pass</t>
+    <t>创建 Booking 时缺少 firstname</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 从 Body 中删除 firstname
+3. 查看响应状态和响应体</t>
+  </si>
+  <si>
+    <t>缺少 firstname，其余字段合法</t>
+  </si>
+  <si>
+    <t>接口应按实际规范校验必填字段；若服务未严格校验，应记录为潜在缺陷并保留实际响应，不要直接判定通过。</t>
   </si>
   <si>
     <t>API-POST-003</t>
   </si>
   <si>
+    <t>创建 Booking 时缺少 bookingdates</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 删除 bookingdates 对象
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>缺少 bookingdates</t>
+  </si>
+  <si>
+    <t>接口应按规范拒绝不完整数据或返回明确错误；若返回成功但数据异常，记录为缺陷候选。</t>
+  </si>
+  <si>
     <t>API-POST-004</t>
   </si>
   <si>
+    <t>创建 Booking 时 totalprice 为字符串</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 将 totalprice 设置为字符串 abc
+3. 查看响应并尝试查询新记录</t>
+  </si>
+  <si>
+    <t>totalprice="abc"</t>
+  </si>
+  <si>
+    <t>接口应进行类型校验并按规范返回处理结果；记录实际返回及持久化结果，不能只依据状态码判断。</t>
+  </si>
+  <si>
     <t>API-POST-005</t>
   </si>
   <si>
+    <t>创建 Booking 时 totalprice 为负数</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 将 totalprice 设置为 -1
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>totalprice=-1</t>
+  </si>
+  <si>
+    <t>若业务规则不允许负价，应拒绝请求或返回校验错误；若接口未定义该规则，记录实际行为供需求确认。</t>
+  </si>
+  <si>
     <t>API-POST-006</t>
   </si>
   <si>
+    <t>创建 Booking 时 depositpaid 为非布尔值</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 将 depositpaid 设置为字符串 yes
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>depositpaid="yes"</t>
+  </si>
+  <si>
+    <t>接口应按字段类型规范校验；记录状态码、响应字段及是否产生异常数据。</t>
+  </si>
+  <si>
     <t>API-POST-007</t>
   </si>
   <si>
+    <t>创建 Booking 时日期格式非法</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /booking
+2. 将 checkin 设置为 2026/10/02
+3. 查看响应及新建数据</t>
+  </si>
+  <si>
+    <t>checkin="2026/10/02"；checkout="2026-10-05"</t>
+  </si>
+  <si>
+    <t>接口应按日期格式规范校验并返回明确结果；若被接受，核对返回值并记录与规范的差异。</t>
+  </si>
+  <si>
     <t>API-POST-008</t>
   </si>
   <si>
-    <t>API-POST-009</t>
-  </si>
-  <si>
-    <t>API-POST-010</t>
-  </si>
-  <si>
-    <t>API-POST-011</t>
-  </si>
-  <si>
-    <t>API-POST-012</t>
-  </si>
-  <si>
-    <t>API-POST-013</t>
-  </si>
-  <si>
-    <t>API-POST-014</t>
-  </si>
-  <si>
-    <t>API-POST-015</t>
-  </si>
-  <si>
-    <t>API-POST-016</t>
-  </si>
-  <si>
-    <t>API-POST-017</t>
-  </si>
-  <si>
-    <t>API-POST-018</t>
+    <t>创建 Booking 时 Content-Type 错误</t>
+  </si>
+  <si>
+    <t>1. 将 Content-Type 改为 text/plain
+2. 发送 JSON 字符串 Body
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>Content-Type: text/plain</t>
+  </si>
+  <si>
+    <t>接口应按服务规范处理不支持的媒体类型，通常返回 4xx；不得产生不可预期的脏数据。</t>
+  </si>
+  <si>
+    <t>API-AUTH-001</t>
+  </si>
+  <si>
+    <t>使用有效凭证获取 Token</t>
+  </si>
+  <si>
+    <t>身份认证</t>
+  </si>
+  <si>
+    <t>POST /auth</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /auth
+2. 查看状态码和响应 JSON
+3. 检查 token 字段</t>
+  </si>
+  <si>
+    <t>{"username":"admin","password":"password123"}</t>
+  </si>
+  <si>
+    <t>返回成功状态并包含非空 token 字段。</t>
+  </si>
+  <si>
+    <t>API-AUTH-002</t>
+  </si>
+  <si>
+    <t>使用错误密码获取 Token</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /auth
+2. 将密码改为错误值
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>username=admin；password=wrong-password</t>
+  </si>
+  <si>
+    <t>认证失败；响应应包含明确失败信息且不应返回有效 token。</t>
+  </si>
+  <si>
+    <t>API-AUTH-003</t>
+  </si>
+  <si>
+    <t>认证请求缺少用户名</t>
+  </si>
+  <si>
+    <t>1. 发送 POST /auth
+2. 删除 username 字段
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>仅传 password=password123</t>
+  </si>
+  <si>
+    <t>认证失败或参数校验失败；不应返回有效 token。</t>
+  </si>
+  <si>
+    <t>API-PUT-001</t>
+  </si>
+  <si>
+    <t>使用有效 Token 完整更新 Booking</t>
+  </si>
+  <si>
+    <t>Booking修改</t>
+  </si>
+  <si>
+    <t>PUT /booking/{id}</t>
+  </si>
+  <si>
+    <t>已创建 Booking；已通过 POST /auth 获取 token</t>
+  </si>
+  <si>
+    <t>1. 创建 Booking 并记录 ID
+2. 获取 token
+3. 发送 PUT /booking/{id}，携带 Cookie: token=...
+4. GET 查询并核对所有更新字段</t>
+  </si>
+  <si>
+    <t>更新为 firstname=Jane、lastname=Doe、totalprice=200、depositpaid=false、日期 2026-11-01 至 2026-11-05、additionalneeds=Late checkout</t>
+  </si>
+  <si>
+    <t>返回 200 OK；查询记录时完整字段更新为新值，未被更新的字段按 PUT 语义及接口规范处理。</t>
+  </si>
+  <si>
+    <t>API-PUT-002</t>
+  </si>
+  <si>
+    <t>PUT 请求不携带 Token</t>
+  </si>
+  <si>
+    <t>已创建 Booking；有有效 ID</t>
+  </si>
+  <si>
+    <t>1. 发送 PUT /booking/{id}
+2. 不携带 Cookie token
+3. 查看响应并重新查询记录</t>
+  </si>
+  <si>
+    <t>合法更新 Body；无 token</t>
+  </si>
+  <si>
+    <t>返回未授权/禁止访问状态（通常为 403）；原记录不应被修改。</t>
+  </si>
+  <si>
+    <t>API-PUT-003</t>
+  </si>
+  <si>
+    <t>使用错误 Token 更新 Booking</t>
+  </si>
+  <si>
+    <t>1. 发送 PUT /booking/{id}
+2. Cookie 中传入错误 token
+3. 查看响应并重新查询记录</t>
+  </si>
+  <si>
+    <t>Cookie: token=invalid-token</t>
+  </si>
+  <si>
+    <t>返回未授权/禁止访问状态；原记录不应被修改。</t>
+  </si>
+  <si>
+    <t>API-PUT-004</t>
+  </si>
+  <si>
+    <t>PUT 更新不存在的 Booking</t>
+  </si>
+  <si>
+    <t>已获取有效 Token</t>
+  </si>
+  <si>
+    <t>1. 发送 PUT /booking/99999999
+2. 携带有效 token
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>不存在的 ID；合法更新 Body</t>
+  </si>
+  <si>
+    <t>返回 404 Not Found 或符合服务规范的错误；不得创建新记录或修改其他记录。</t>
+  </si>
+  <si>
+    <t>API-PATCH-001</t>
+  </si>
+  <si>
+    <t>使用有效 Token 局部更新单个字段</t>
+  </si>
+  <si>
+    <t>Booking局部修改</t>
+  </si>
+  <si>
+    <t>PATCH /booking/{id}</t>
+  </si>
+  <si>
+    <t>已创建 Booking；已获取有效 Token</t>
+  </si>
+  <si>
+    <t>1. 记录更新前数据
+2. 发送 PATCH /booking/{id}
+3. 仅传 firstname 字段
+4. GET 查询并对比</t>
+  </si>
+  <si>
+    <t>{"firstname":"Alice"}</t>
+  </si>
+  <si>
+    <t>返回成功状态；firstname 更新为 Alice，其余字段保持原值。</t>
+  </si>
+  <si>
+    <t>API-PATCH-002</t>
+  </si>
+  <si>
+    <t>PATCH 不携带 Token</t>
+  </si>
+  <si>
+    <t>1. 发送 PATCH /booking/{id}
+2. 不携带 token
+3. 查看响应并核对记录</t>
+  </si>
+  <si>
+    <t>合法局部更新 Body；无 token</t>
+  </si>
+  <si>
+    <t>返回未授权/禁止访问状态；记录不应被修改。</t>
+  </si>
+  <si>
+    <t>API-PATCH-003</t>
+  </si>
+  <si>
+    <t>PATCH 传入空 Body</t>
+  </si>
+  <si>
+    <t>1. 发送空 JSON 对象 {}
+2. 查看响应
+3. GET 查询记录</t>
+  </si>
+  <si>
+    <t>{}</t>
+  </si>
+  <si>
+    <t>接口应按规范返回成功或校验结果；若成功，原字段应保持不变。记录实际行为。</t>
+  </si>
+  <si>
+    <t>API-DELETE-001</t>
+  </si>
+  <si>
+    <t>使用有效 Token 删除 Booking</t>
+  </si>
+  <si>
+    <t>Booking删除</t>
+  </si>
+  <si>
+    <t>DELETE /booking/{id}</t>
+  </si>
+  <si>
+    <t>1. 创建 Booking 并记录 ID
+2. 发送 DELETE /booking/{id} 并携带 token
+3. 查看响应
+4. GET 查询该 ID</t>
+  </si>
+  <si>
+    <t>Cookie: token=&lt;有效 token&gt;</t>
+  </si>
+  <si>
+    <t>删除请求返回成功状态（通常为 201 Created）；之后查询该 ID 应返回 404，证明记录已删除。</t>
+  </si>
+  <si>
+    <t>API-DELETE-002</t>
+  </si>
+  <si>
+    <t>DELETE 请求不携带 Token</t>
+  </si>
+  <si>
+    <t>1. 发送 DELETE /booking/{id}
+2. 不携带 token
+3. 查看响应
+4. GET 查询记录</t>
+  </si>
+  <si>
+    <t>无 token</t>
+  </si>
+  <si>
+    <t>返回未授权/禁止访问状态；记录仍然存在。</t>
+  </si>
+  <si>
+    <t>API-DELETE-003</t>
+  </si>
+  <si>
+    <t>删除不存在的 Booking</t>
+  </si>
+  <si>
+    <t>1. 发送 DELETE /booking/99999999
+2. 携带有效 token
+3. 查看响应</t>
+  </si>
+  <si>
+    <t>不存在的 ID</t>
+  </si>
+  <si>
+    <t>返回符合接口规范的错误状态；不应影响其他记录。</t>
+  </si>
+  <si>
+    <t>API-DELETE-004</t>
+  </si>
+  <si>
+    <t>重复删除同一 Booking</t>
+  </si>
+  <si>
+    <t>已创建 Booking；已获取有效 Token；首次删除成功</t>
+  </si>
+  <si>
+    <t>1. 首次删除该 Booking 并确认成功
+2. 再次发送相同 DELETE 请求
+3. 查看第二次响应</t>
+  </si>
+  <si>
+    <t>同一 bookingid</t>
+  </si>
+  <si>
+    <t>第二次删除应返回未找到或符合接口规范的结果；不应影响其他记录。</t>
+  </si>
+  <si>
+    <t>API-SEC-001</t>
+  </si>
+  <si>
+    <t>请求不存在的路由</t>
+  </si>
+  <si>
+    <t>接口通用/异常处理</t>
+  </si>
+  <si>
+    <t>GET /not-a-real-endpoint</t>
+  </si>
+  <si>
+    <t>1. 发送 GET /not-a-real-endpoint
+2. 查看状态码和响应内容</t>
+  </si>
+  <si>
+    <t>返回 404 Not Found 或符合路由规范的错误响应；不得返回误导性成功结果。</t>
+  </si>
+  <si>
+    <t>API-SEC-002</t>
+  </si>
+  <si>
+    <t>检查响应是否泄露敏感信息</t>
+  </si>
+  <si>
+    <t>接口通用/安全</t>
+  </si>
+  <si>
+    <t>GET /booking/{id}；POST /auth</t>
+  </si>
+  <si>
+    <t>服务可访问；存在有效 ID</t>
+  </si>
+  <si>
+    <t>1. 调用查询接口和认证失败接口
+2. 检查响应体及错误信息
+3. 检查是否包含密码、内部堆栈或密钥</t>
+  </si>
+  <si>
+    <t>合法查询数据；错误密码</t>
+  </si>
+  <si>
+    <t>响应不应泄露密码、密钥、服务器堆栈等敏感信息；只返回业务所需字段及合理错误信息。</t>
+  </si>
+  <si>
+    <t>API-DATA-001</t>
+  </si>
+  <si>
+    <t>创建后更新再删除的完整流程</t>
+  </si>
+  <si>
+    <t>端到端流程</t>
+  </si>
+  <si>
+    <t>POST → GET → PUT/PATCH → DELETE</t>
+  </si>
+  <si>
+    <t>服务可访问；可获取 Token</t>
+  </si>
+  <si>
+    <t>1. POST 创建记录
+2. GET 查询核对
+3. PUT 或 PATCH 更新
+4. GET 验证更新
+5. DELETE 删除
+6. GET 验证不存在</t>
+  </si>
+  <si>
+    <t>使用本用例独立生成的 Booking 数据和有效 token</t>
+  </si>
+  <si>
+    <t>各步骤状态码符合接口规范；数据在创建、查询、更新、删除各阶段状态正确，无残留记录。</t>
+  </si>
+  <si>
+    <t>Restful Booker API 测试用例执行说明</t>
+  </si>
+  <si>
+    <t>项目地址</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com</t>
+  </si>
+  <si>
+    <t>测试工具</t>
+  </si>
+  <si>
+    <t>Postman；可结合 Newman 命令行运行和生成报告</t>
+  </si>
+  <si>
+    <t>用例范围</t>
+  </si>
+  <si>
+    <t>健康检查、Booking 查询/创建/认证/完整更新/局部更新/删除、异常与端到端流程</t>
+  </si>
+  <si>
+    <t>执行前准备</t>
+  </si>
+  <si>
+    <t>确认服务可访问；创建/更新/删除用例建议使用自己创建的 bookingid；认证用例使用接口文档提供的测试凭证。</t>
+  </si>
+  <si>
+    <t>动态数据提醒</t>
+  </si>
+  <si>
+    <t>bookingid 是动态生成的，不要固定写死；先执行 POST 创建，再把返回的 bookingid 用于后续 GET/PUT/PATCH/DELETE。</t>
+  </si>
+  <si>
+    <t>Token 提醒</t>
+  </si>
+  <si>
+    <t>POST /auth 成功后读取 token；修改和删除请求按接口要求设置 Cookie: token=&lt;token&gt;。</t>
+  </si>
+  <si>
+    <t>预期结果说明</t>
+  </si>
+  <si>
+    <t>部分异常参数的精确行为可能取决于当前 Restful Booker 服务版本。若接口规范没有明确规定，按“记录实际行为、对照规范判定”执行，不要只凭通用预期判缺陷。</t>
+  </si>
+  <si>
+    <t>实际结果填写</t>
+  </si>
+  <si>
+    <t>每次执行后记录实际状态码、关键响应字段、是否创建/修改/删除成功；失败时附 Postman 响应或报告截图。</t>
+  </si>
+  <si>
+    <t>测试结论填写</t>
+  </si>
+  <si>
+    <t>Pass：实际结果符合预期；Fail：与预期不符且可复现；Blocked：环境或前置条件阻塞；待执行：尚未执行。</t>
+  </si>
+  <si>
+    <t>用例数量</t>
+  </si>
+  <si>
+    <t>33 条用例</t>
   </si>
 </sst>
 </file>
@@ -234,13 +858,31 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -261,24 +903,9 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.3"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.3"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -425,7 +1052,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -434,6 +1061,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -637,12 +1276,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E1F2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E1F2"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -846,76 +1500,70 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="13">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="14">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="15">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="17" borderId="0">
@@ -924,10 +1572,10 @@
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="0">
@@ -936,10 +1584,10 @@
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="25" borderId="0">
@@ -948,10 +1596,10 @@
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="29" borderId="0">
@@ -960,10 +1608,10 @@
     <xf numFmtId="0" fontId="24" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0">
@@ -972,52 +1620,51 @@
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1330,409 +1977,1357 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="34.2222222222222" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="16.3333333333333" customWidth="1"/>
-    <col min="5" max="6" width="18.6666666666667" customWidth="1"/>
-    <col min="7" max="7" width="51.6666666666667" customWidth="1"/>
-    <col min="8" max="8" width="48.5555555555556" customWidth="1"/>
-    <col min="9" max="9" width="29.8888888888889" customWidth="1"/>
-    <col min="10" max="10" width="38.8888888888889" customWidth="1"/>
-    <col min="11" max="11" width="12.8888888888889" customWidth="1"/>
+    <col min="1" max="1" width="17" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="6" width="27" style="1" customWidth="1"/>
+    <col min="7" max="7" width="44" style="1" customWidth="1"/>
+    <col min="8" max="8" width="42" style="1" customWidth="1"/>
+    <col min="9" max="9" width="48" style="1" customWidth="1"/>
+    <col min="10" max="10" width="28" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:11">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" ht="46.8" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" ht="86.4" spans="1:11">
-      <c r="A3" s="7" t="s">
+    <row r="3" ht="72" customHeight="1" spans="1:11">
+      <c r="A3" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="9" t="s">
+    </row>
+    <row r="4" ht="72" customHeight="1" spans="1:11">
+      <c r="A4" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" ht="158.4" spans="1:11">
-      <c r="A4" s="7" t="s">
+      <c r="B4" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="8" t="s">
+      <c r="F4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="G4" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="H4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1" spans="1:11">
+      <c r="A5" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="B5" s="12" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" ht="28.8" spans="1:11">
-      <c r="A5" s="7" t="s">
+      <c r="C5" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="9"/>
-    </row>
-    <row r="6" ht="28.8" spans="1:11">
-      <c r="A6" s="7" t="s">
+      <c r="F5" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" ht="28.8" spans="1:11">
-      <c r="A7" s="7" t="s">
+      <c r="G5" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="9"/>
-    </row>
-    <row r="8" ht="28.8" spans="1:11">
-      <c r="A8" s="7" t="s">
+      <c r="H5" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" ht="28.8" spans="1:11">
-      <c r="A9" s="7" t="s">
+      <c r="I5" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="9"/>
-    </row>
-    <row r="10" ht="28.8" spans="1:11">
-      <c r="A10" s="7" t="s">
+      <c r="J5" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:11">
+      <c r="A6" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" ht="28.8" spans="1:11">
-      <c r="A11" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" ht="28.8" spans="1:11">
-      <c r="A12" s="7" t="s">
+      <c r="C6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" ht="28.8" spans="1:11">
-      <c r="A13" s="7" t="s">
+      <c r="E6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" ht="28.8" spans="1:11">
-      <c r="A14" s="7" t="s">
+      <c r="H6" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" ht="28.8" spans="1:11">
-      <c r="A15" s="7" t="s">
+      <c r="I6" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" ht="28.8" spans="1:11">
-      <c r="A16" s="7" t="s">
+      <c r="J6" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1" spans="1:11">
+      <c r="A7" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" ht="28.8" spans="1:11">
-      <c r="A17" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" ht="28.8" spans="1:11">
-      <c r="A18" s="7" t="s">
+      <c r="C7" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" ht="28.8" spans="1:11">
-      <c r="A19" s="7" t="s">
+      <c r="E7" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" ht="28.8" spans="1:11">
-      <c r="A20" s="7" t="s">
+      <c r="H7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
+      <c r="I7" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1" spans="1:11">
+      <c r="A8" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1" spans="1:11">
+      <c r="A9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1" spans="1:11">
+      <c r="A10" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1" spans="1:11">
+      <c r="A11" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1" spans="1:11">
+      <c r="A12" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1" spans="1:11">
+      <c r="A13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1" spans="1:11">
+      <c r="A14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1" spans="1:11">
+      <c r="A15" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1" spans="1:11">
+      <c r="A16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1" spans="1:11">
+      <c r="A17" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1" spans="1:11">
+      <c r="A18" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1" spans="1:11">
+      <c r="A19" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="K19" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" ht="72" customHeight="1" spans="1:11">
+      <c r="A20" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1" spans="1:11">
+      <c r="A21" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="I21" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1" spans="1:11">
+      <c r="A22" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1" spans="1:11">
+      <c r="A23" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K23" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1" spans="1:11">
+      <c r="A24" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1" spans="1:11">
+      <c r="A25" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1" spans="1:11">
+      <c r="A26" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1" spans="1:11">
+      <c r="A27" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" ht="72" customHeight="1" spans="1:11">
+      <c r="A28" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1" spans="1:11">
+      <c r="A29" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="K29" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1" spans="1:11">
+      <c r="A30" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="K30" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1" spans="1:11">
+      <c r="A31" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="K31" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1" spans="1:11">
+      <c r="A32" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="K32" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1" spans="1:11">
+      <c r="A33" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="K33" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1" spans="1:11">
+      <c r="A34" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="K34" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1" spans="1:11">
+      <c r="A35" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="K35" s="12" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K35" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="22" style="1" customWidth="1"/>
+    <col min="2" max="2" width="105" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20.4" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1" spans="1:2">
+      <c r="A2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1" spans="1:2">
+      <c r="A3" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1" spans="1:2">
+      <c r="A4" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1" spans="1:2">
+      <c r="A5" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1" spans="1:2">
+      <c r="A6" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1" spans="1:2">
+      <c r="A7" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1" spans="1:2">
+      <c r="A8" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1" spans="1:2">
+      <c r="A9" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1" spans="1:2">
+      <c r="A10" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1" spans="1:2">
+      <c r="A11" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>